<commit_message>
add doi to README
</commit_message>
<xml_diff>
--- a/supplements/S1_change_detection_sensitivity.xlsx
+++ b/supplements/S1_change_detection_sensitivity.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="README_summary" sheetId="1" state="visible" r:id="rId3"/>
@@ -83,35 +83,7 @@
     <t xml:space="preserve">Removed segments (n)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Baseline (10 m buffer, 15 m realignment, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">10 m minimum segment)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Baseline (10 m buffer, 15 m realignment, 10 m minimum segment))</t>
   </si>
   <si>
     <t xml:space="preserve">Buffer = 5 m</t>
@@ -139,7 +111,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,12 +140,6 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -481,11 +447,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="68432327"/>
-        <c:axId val="8991331"/>
+        <c:axId val="61341206"/>
+        <c:axId val="14801347"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="68432327"/>
+        <c:axId val="61341206"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -551,7 +517,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8991331"/>
+        <c:crossAx val="14801347"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -559,7 +525,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8991331"/>
+        <c:axId val="14801347"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -635,7 +601,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68432327"/>
+        <c:crossAx val="61341206"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -698,9 +664,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>585360</xdr:colOff>
+      <xdr:colOff>585000</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>14400</xdr:rowOff>
+      <xdr:rowOff>14040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -709,7 +675,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="14961960" y="190440"/>
-        <a:ext cx="5399280" cy="2699280"/>
+        <a:ext cx="5398920" cy="2698920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">

</xml_diff>